<commit_message>
Fixed template metadata variable names
</commit_message>
<xml_diff>
--- a/MARMOT_Metadata.xlsx
+++ b/MARMOT_Metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peterleary/Desktop/FGCZ/MARMOT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15AF043D-402B-2248-96BB-4D0A8FAE27FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55FF4185-5194-2C45-8321-E6CB151EE7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3460" yWindow="2760" windowWidth="39400" windowHeight="21660" xr2:uid="{9C611E3C-4644-F449-9441-E60F328909FC}"/>
   </bookViews>
@@ -324,9 +324,6 @@
     <t>runQC</t>
   </si>
   <si>
-    <t>removeFromQC</t>
-  </si>
-  <si>
     <t>useQC</t>
   </si>
   <si>
@@ -496,6 +493,9 @@
   </si>
   <si>
     <t>Select a ggplot theme to use. Marmots like prism.</t>
+  </si>
+  <si>
+    <t>metricsQC</t>
   </si>
 </sst>
 </file>
@@ -1317,13 +1317,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C1" s="5" t="s">
         <v>103</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -1334,7 +1334,7 @@
         <v>1000</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -1342,10 +1342,10 @@
         <v>84</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1353,10 +1353,10 @@
         <v>85</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -1364,10 +1364,10 @@
         <v>86</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -1378,7 +1378,7 @@
         <v>20</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -1386,10 +1386,10 @@
         <v>88</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -1400,7 +1400,7 @@
         <v>47</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="B9" s="18"/>
       <c r="C9" s="19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -1420,115 +1420,115 @@
         <v>1</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="20" t="s">
-        <v>92</v>
+        <v>149</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="20" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B12" s="21" t="b">
         <v>0</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="23" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B13" s="24"/>
       <c r="C13" s="25" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B14" s="24" t="b">
         <v>1</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="23" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B15" s="24" t="b">
         <v>0</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="23" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B16" s="24" t="b">
         <v>1</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="23" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B17" s="24">
         <v>4</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B18" s="24">
         <v>6</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="23" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -1536,10 +1536,10 @@
         <v>81</v>
       </c>
       <c r="B21" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="C21" s="28" t="s">
         <v>139</v>
-      </c>
-      <c r="C21" s="28" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -1547,10 +1547,10 @@
         <v>82</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -2194,93 +2194,93 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B1" t="s">
         <v>47</v>
       </c>
       <c r="C1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D1" t="b">
         <v>1</v>
       </c>
       <c r="E1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B2" t="s">
         <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="E5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>